<commit_message>
fix: paginacion completa en descarga Linkaform (>1000 registros) y acumulacion de celdas en reporte diario
</commit_message>
<xml_diff>
--- a/data/CANTIDADES_MATERIALES_RECIBIDOS_ACTUALIZADO.xlsx
+++ b/data/CANTIDADES_MATERIALES_RECIBIDOS_ACTUALIZADO.xlsx
@@ -38360,7 +38360,9 @@
       <c r="Q9" s="100" t="n"/>
       <c r="R9" s="22" t="n"/>
       <c r="S9" s="100" t="n"/>
-      <c r="T9" s="22" t="n"/>
+      <c r="T9" s="22" t="n">
+        <v>416</v>
+      </c>
       <c r="U9" s="100" t="n"/>
       <c r="V9" s="22" t="n"/>
       <c r="W9" s="100" t="n"/>
@@ -62101,7 +62103,9 @@
       </c>
       <c r="S261" s="22" t="n"/>
       <c r="T261" s="61" t="n"/>
-      <c r="U261" s="22" t="n"/>
+      <c r="U261" s="22" t="n">
+        <v>380</v>
+      </c>
       <c r="V261" s="61" t="n"/>
       <c r="W261" s="22" t="n"/>
       <c r="X261" s="61" t="n"/>
@@ -64237,7 +64241,9 @@
       <c r="R299" s="61" t="n"/>
       <c r="S299" s="22" t="n"/>
       <c r="T299" s="61" t="n"/>
-      <c r="U299" s="22" t="n"/>
+      <c r="U299" s="22" t="n">
+        <v>1</v>
+      </c>
       <c r="V299" s="61" t="n"/>
       <c r="W299" s="22" t="n"/>
       <c r="X299" s="61" t="n"/>
@@ -66255,7 +66261,9 @@
       <c r="R335" s="61" t="n"/>
       <c r="S335" s="22" t="n"/>
       <c r="T335" s="61" t="n"/>
-      <c r="U335" s="22" t="n"/>
+      <c r="U335" s="22" t="n">
+        <v>110</v>
+      </c>
       <c r="V335" s="61" t="n"/>
       <c r="W335" s="22" t="n"/>
       <c r="X335" s="61" t="n"/>

</xml_diff>